<commit_message>
Add experiment 3 in private folder
</commit_message>
<xml_diff>
--- a/private/OUTPUT_test1.xlsx
+++ b/private/OUTPUT_test1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\00040628\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\00040628\LocalData\GitHub\14224ontologies_public\private\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4490181A-C60F-4F2D-A37E-31CDDD8BB0FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1EFE23-B471-4E61-A769-94597F83CB2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9585" yWindow="-20415" windowWidth="23775" windowHeight="17820" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1251,69 +1251,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1329,27 +1266,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1419,7 +1335,42 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1440,7 +1391,56 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1536,11 +1536,61 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>311150</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4974DE1-5BAD-78D5-EA9A-AED27738CFFB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="6350000" cy="17462500"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5765,17 +5815,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q19">
-    <cfRule type="cellIs" dxfId="31" priority="102" operator="between">
-      <formula>"H10"</formula>
-      <formula>"H17"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="104" operator="between">
+    <cfRule type="cellIs" dxfId="31" priority="104" operator="between">
       <formula>"M6"</formula>
       <formula>"M9"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="103" operator="between">
+    <cfRule type="cellIs" dxfId="30" priority="103" operator="between">
       <formula>"L1"</formula>
       <formula>"L5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="102" operator="between">
+      <formula>"H10"</formula>
+      <formula>"H17"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="28" priority="101" operator="between">
       <formula>"E19"</formula>
@@ -5819,53 +5869,53 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q29">
-    <cfRule type="cellIs" dxfId="19" priority="92" operator="between">
-      <formula>"M6"</formula>
-      <formula>"M9"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="89" operator="between">
+    <cfRule type="cellIs" dxfId="19" priority="89" operator="between">
       <formula>"E19"</formula>
       <formula>"E25"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="90" operator="between">
+    <cfRule type="cellIs" dxfId="18" priority="90" operator="between">
       <formula>"H10"</formula>
       <formula>"H17"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="91" operator="between">
+    <cfRule type="cellIs" dxfId="17" priority="91" operator="between">
       <formula>"L1"</formula>
       <formula>"L5"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R22">
-    <cfRule type="cellIs" dxfId="15" priority="87" operator="between">
-      <formula>"L1"</formula>
-      <formula>"L5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="86" operator="between">
-      <formula>"H10"</formula>
-      <formula>"H17"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="85" operator="between">
-      <formula>"E19"</formula>
-      <formula>"E25"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="88" operator="between">
+    <cfRule type="cellIs" dxfId="16" priority="92" operator="between">
       <formula>"M6"</formula>
       <formula>"M9"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U52">
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="between">
+  <conditionalFormatting sqref="R22">
+    <cfRule type="cellIs" dxfId="15" priority="88" operator="between">
+      <formula>"M6"</formula>
+      <formula>"M9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="87" operator="between">
+      <formula>"L1"</formula>
+      <formula>"L5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="86" operator="between">
       <formula>"H10"</formula>
       <formula>"H17"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="4" operator="between">
+    <cfRule type="cellIs" dxfId="12" priority="85" operator="between">
+      <formula>"E19"</formula>
+      <formula>"E25"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U2:U52">
+    <cfRule type="cellIs" dxfId="11" priority="4" operator="between">
       <formula>"M6"</formula>
       <formula>"M9"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="10" priority="3" operator="between">
       <formula>"L1"</formula>
       <formula>"L5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="between">
+      <formula>"H10"</formula>
+      <formula>"H17"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="8" priority="1" operator="between">
       <formula>"E19"</formula>
@@ -5873,21 +5923,21 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U55:U56">
-    <cfRule type="cellIs" dxfId="7" priority="18" operator="between">
+    <cfRule type="cellIs" dxfId="7" priority="20" operator="between">
+      <formula>"M6"</formula>
+      <formula>"M9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="19" operator="between">
+      <formula>"L1"</formula>
+      <formula>"L5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="18" operator="between">
       <formula>"H10"</formula>
       <formula>"H17"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="17" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="17" operator="between">
       <formula>"E19"</formula>
       <formula>"E25"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="20" operator="between">
-      <formula>"M6"</formula>
-      <formula>"M9"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="19" operator="between">
-      <formula>"L1"</formula>
-      <formula>"L5"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U59:U60">

</xml_diff>